<commit_message>
Add modern Dark Mode GUI, Show Chrome toggle, and PyInstaller standalone build
</commit_message>
<xml_diff>
--- a/oppo_results.xlsx
+++ b/oppo_results.xlsx
@@ -613,7 +613,7 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -903,7 +903,7 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1495,7 @@
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-15 01:32:15</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1855,7 @@
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J24" s="4" t="n"/>
+      <c r="J24" s="4" t="inlineStr"/>
       <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J25" s="4" t="n"/>
+      <c r="J25" s="4" t="inlineStr"/>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1971,7 +1971,7 @@
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2021,7 +2021,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J26" s="4" t="n"/>
+      <c r="J26" s="4" t="inlineStr"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J27" s="4" t="n"/>
+      <c r="J27" s="4" t="inlineStr"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J28" s="4" t="n"/>
+      <c r="J28" s="4" t="inlineStr"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2207,7 @@
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2257,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J30" s="4" t="n"/>
+      <c r="J30" s="4" t="inlineStr"/>
       <c r="K30" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2315,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J31" s="4" t="n"/>
+      <c r="J31" s="4" t="inlineStr"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J33" s="4" t="n"/>
+      <c r="J33" s="4" t="inlineStr"/>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2443,7 +2443,7 @@
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J36" s="4" t="n"/>
+      <c r="J36" s="4" t="inlineStr"/>
       <c r="K36" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2749,7 +2749,7 @@
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2759,19 +2759,19 @@
           <t>864223086198994</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Not Activated</t>
+          <t>Pending Sync</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Not Activated</t>
+          <t>The activation time has been transferred to the system. Please check again after 7 days.</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2861,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J40" s="4" t="n"/>
+      <c r="J40" s="4" t="inlineStr"/>
       <c r="K40" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="L40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2919,7 +2919,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J41" s="4" t="n"/>
+      <c r="J41" s="4" t="inlineStr"/>
       <c r="K41" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>
@@ -2937,19 +2937,19 @@
           <t>864223084794877</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Not Activated</t>
+          <t>1791323329000</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Not Activated</t>
+          <t>1791323329000</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="L42" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12 23:31:24</t>
+          <t>2026-10-15 01:38:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Format activation dates to DD-MM-YYYY (UTC+3), update dashboard Total Serials to count input file, and synchronize Total in Sheet
</commit_message>
<xml_diff>
--- a/oppo_results.xlsx
+++ b/oppo_results.xlsx
@@ -485,14 +485,14 @@
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="92" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
   </cols>
@@ -605,7 +605,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="n"/>
       <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -663,7 +663,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -721,7 +721,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="J4" s="4" t="n"/>
       <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -779,7 +779,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="n"/>
       <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -837,7 +837,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="n"/>
       <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -895,7 +895,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -920,12 +920,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>1790368620000</t>
+          <t>25-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1790368620000</t>
+          <t>25-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>1826656620000</t>
+          <t>19-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1015,7 +1015,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1073,7 +1073,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="n"/>
       <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1131,7 +1131,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1189,7 +1189,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="n"/>
       <c r="K12" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1247,7 +1247,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1272,12 +1272,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>1791028220000</t>
+          <t>03-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1791028220000</t>
+          <t>03-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>1827316220000</t>
+          <t>27-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
@@ -1367,7 +1367,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="n"/>
       <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1392,12 +1392,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>1791142738000</t>
+          <t>04-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>1791142738000</t>
+          <t>04-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>1827430738000</t>
+          <t>28-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -1487,7 +1487,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1545,7 +1545,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="J18" s="4" t="n"/>
       <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>1827783421000</t>
+          <t>03-12-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
@@ -1665,7 +1665,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="n"/>
       <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1723,7 +1723,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1748,12 +1748,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>1791224840000</t>
+          <t>05-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1791224840000</t>
+          <t>05-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>1827512840000</t>
+          <t>29-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
@@ -1810,12 +1810,12 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>1790538429000</t>
+          <t>27-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1790538429000</t>
+          <t>27-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>1826826429000</t>
+          <t>21-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
@@ -1905,7 +1905,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -1963,7 +1963,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2021,7 +2021,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2079,7 +2079,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="n"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2137,7 +2137,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
+      <c r="J28" s="4" t="n"/>
       <c r="K28" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2162,12 +2162,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>1791226324000</t>
+          <t>05-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1791226324000</t>
+          <t>05-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>1827514324000</t>
+          <t>29-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K29" s="4" t="inlineStr">
@@ -2257,7 +2257,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="n"/>
       <c r="K30" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2315,7 +2315,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2340,12 +2340,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>1790612057000</t>
+          <t>28-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1790612057000</t>
+          <t>28-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>1826900057000</t>
+          <t>22-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K32" s="4" t="inlineStr">
@@ -2435,7 +2435,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
+      <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2460,12 +2460,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>1790520479000</t>
+          <t>27-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1790520479000</t>
+          <t>27-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>1826808479000</t>
+          <t>21-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K34" s="4" t="inlineStr">
@@ -2522,12 +2522,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>1790656059000</t>
+          <t>29-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1790656059000</t>
+          <t>29-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="J35" s="4" t="inlineStr">
         <is>
-          <t>1826944059000</t>
+          <t>23-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
@@ -2617,7 +2617,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="n"/>
       <c r="K36" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2642,12 +2642,12 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>1790361696000</t>
+          <t>25-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1790361696000</t>
+          <t>25-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>1826649696000</t>
+          <t>19-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K37" s="4" t="inlineStr">
@@ -2704,12 +2704,12 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>1790955768000</t>
+          <t>02-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>1790955768000</t>
+          <t>02-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>1827243768000</t>
+          <t>26-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K38" s="4" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="J39" s="4" t="inlineStr">
         <is>
-          <t>1827956901000</t>
+          <t>05-12-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K39" s="4" t="inlineStr">
@@ -2861,7 +2861,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="n"/>
       <c r="K40" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2919,7 +2919,7 @@
           <t>UA</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="n"/>
       <c r="K41" s="4" t="inlineStr">
         <is>
           <t>Found</t>
@@ -2944,12 +2944,12 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>1791323329000</t>
+          <t>07-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>1791323329000</t>
+          <t>07-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>1827611329000</t>
+          <t>01-12-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K42" s="4" t="inlineStr">
@@ -3064,12 +3064,12 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>1790714144000</t>
+          <t>29-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>1790714144000</t>
+          <t>29-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>1827002144000</t>
+          <t>23-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K44" s="4" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>1828111312000</t>
+          <t>06-12-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K45" s="4" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="J57" s="4" t="inlineStr">
         <is>
-          <t>1828019415000</t>
+          <t>05-12-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K57" s="4" t="inlineStr">
@@ -3923,7 +3923,7 @@
       </c>
       <c r="J58" s="4" t="inlineStr">
         <is>
-          <t>1827596869000</t>
+          <t>30-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K58" s="4" t="inlineStr">
@@ -4066,12 +4066,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>1790889713000</t>
+          <t>02-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>1790889713000</t>
+          <t>02-10-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="J61" s="4" t="inlineStr">
         <is>
-          <t>1827177713000</t>
+          <t>26-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K61" s="4" t="inlineStr">
@@ -4186,12 +4186,12 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>1790606334000</t>
+          <t>28-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>1790606334000</t>
+          <t>28-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t>1826894334000</t>
+          <t>22-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K63" s="4" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>1790583066000</t>
+          <t>28-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>1790583066000</t>
+          <t>28-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="J64" s="4" t="inlineStr">
         <is>
-          <t>1826871066000</t>
+          <t>22-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K64" s="4" t="inlineStr">
@@ -4310,12 +4310,12 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>1790675403000</t>
+          <t>29-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>1790675403000</t>
+          <t>29-09-2026 (UTC+3)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="J65" s="4" t="inlineStr">
         <is>
-          <t>1826963403000</t>
+          <t>23-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K65" s="4" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="J68" s="4" t="inlineStr">
         <is>
-          <t>1827590211000</t>
+          <t>30-11-2027 (UTC+3)</t>
         </is>
       </c>
       <c r="K68" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add Linux launcher, live timer & ETA, parallel multi-threading, and optimized captcha trajectory
</commit_message>
<xml_diff>
--- a/oppo_results.xlsx
+++ b/oppo_results.xlsx
@@ -37,7 +37,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +68,12 @@
         <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -95,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -113,6 +119,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -480,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -493,7 +502,7 @@
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
     <col width="23" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
@@ -4537,6 +4546,484 @@
         </is>
       </c>
     </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>863546086739990</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>08-10-2026 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>08-10-2026 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>02-12-2027 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>863546086744776</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="n"/>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>863546086745674</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="n"/>
+      <c r="K71" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L71" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>863546086746839</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Pending Sync</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>The activation time has been transferred to the system. Please check again after 7 days.</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>06-12-2027 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>863546086746854</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="n"/>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>863546086746953</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Not Activated</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="n"/>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L74" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>863546086749718</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>27-09-2026 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>27-09-2026 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>OPPO A6</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>8GB+256GB</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Aurora Gold</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>CPH2817</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>21-11-2027 (UTC+3)</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>863546086748991</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="n"/>
+      <c r="D76" s="2" t="n"/>
+      <c r="E76" s="2" t="n"/>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="2" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
+      <c r="J76" s="4" t="n"/>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>Captcha Failed</t>
+        </is>
+      </c>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>863546086748215</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="n"/>
+      <c r="D77" s="2" t="n"/>
+      <c r="E77" s="2" t="n"/>
+      <c r="F77" s="4" t="n"/>
+      <c r="G77" s="2" t="n"/>
+      <c r="H77" s="4" t="n"/>
+      <c r="I77" s="4" t="n"/>
+      <c r="J77" s="4" t="n"/>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-17 21:53:04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>